<commit_message>
Bedarfsliste 0.4: Bedarfsseite neu aufgebaut
- Liste: über der Tabelle nur Suche und Stichwort
- Kopf: Name und Gliederung direkt änderbar, Summe hinter einem Strich mit
  Schätzung/laut Angebot; rechts „⋯“ (zurückstellen, verwerfen, archivieren) und Löschen
- rechte Spalte: Freigaben, Unterlagen und Ordner mit Kreisen (grün ✓, gelb …, rot ✗),
  Klick auf den Kreis bietet die Stände an
- Förderplan ohne Kästen: Name als Überschrift mit Stift, Summe mit Anteil, Stand-Knopf
  mit Fristen, Einschätzung als fünf Punkte, Pro und Contra (auch in der Excel-Vorlage)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -299,12 +299,12 @@
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warum passt das?</t>
+          <t xml:space="preserve">Pro – warum passt das?</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Knackpunkte</t>
+          <t xml:space="preserve">Contra – Knackpunkte</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warum passt das?</t>
+          <t xml:space="preserve">Pro – warum passt das?</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Knackpunkte</t>
+          <t xml:space="preserve">Contra – Knackpunkte</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Bedarfsliste 0.15: Förderrecherche mit Copilot
- Knopf „Recherche mit Copilot“ im Förderplan: Excel anlegen, Prompt kopieren, Ergebnis übernehmen
- Excel im Unterordner „Förderrecherche“ (mit Ordner) oder als Download; beschreibt Bedarf mit Finanzierung, Förderer mit Stand, Kartei-Auszug je Gliederung ohne Kontaktdaten
- Prompt mit Auftrag, Region, Umfang und Format, vorher anpassbar
- Vorschläge mit Begründung, Hinweis „ohne Quelle“ und Summe der neu ausgewählten Förderer

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -155,22 +155,23 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="32" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="48" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="48" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
-    <col min="16" max="16" width="36" customWidth="1"/>
-    <col min="17" max="17" width="30" customWidth="1"/>
+    <col min="15" max="15" width="48" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="36" customWidth="1"/>
+    <col min="18" max="18" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -183,7 +184,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Je möglichem Förderer eine Zeile ausfüllen. Spaltenüberschriften und Blattnamen nicht ändern. Was in jede Spalte gehört, steht im Blatt „Anleitung“. Danach in der Bedarfsliste „Aus Excel übernehmen“ wählen.</t>
+          <t xml:space="preserve">Je möglichem Förderer eine Zeile ausfüllen. Spaltenüberschriften und Blattnamen nicht ändern. Auftrag, Umfang und was in jede Spalte gehört, stehen im Blatt „Anleitung“. Danach in der Bedarfsliste „Excel übernehmen“ wählen.</t>
         </is>
       </c>
     </row>
@@ -215,15 +216,15 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deadline</t>
+          <t xml:space="preserve">Eigenmittel (€)</t>
         </is>
       </c>
       <c r="B7" s="4"/>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beschreibung</t>
+          <t xml:space="preserve">Schon zugesagt (€)</t>
         </is>
       </c>
       <c r="B8" s="4"/>
@@ -231,192 +232,135 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Noch offen (€)</t>
+        </is>
+      </c>
+      <c r="B9" s="4"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deadline</t>
+        </is>
+      </c>
+      <c r="B10" s="4"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stichwort oder Fördertopf</t>
+        </is>
+      </c>
+      <c r="B11" s="4"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beschreibung</t>
+        </is>
+      </c>
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Kennung</t>
         </is>
       </c>
-      <c r="B9" s="5"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B13" s="5"/>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Förderer</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stand in der Bedarfsliste</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Art</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Antragsweg</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Ansprechperson oder Portal</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">E-Mail</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Telefon</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Website oder Portal-Link</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Antragsfrist</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Weitere Fristen und Termine</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Erwartete Summe (€)</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Übliche Fördersumme</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Eigenanteil gefordert</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Pro – warum passt das?</t>
         </is>
       </c>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Contra – Knackpunkte</t>
         </is>
       </c>
-      <c r="O10" s="6" t="inlineStr">
+      <c r="P15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Einschätzung</t>
         </is>
       </c>
-      <c r="P10" s="6" t="inlineStr">
+      <c r="Q15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Quellen</t>
         </is>
       </c>
-      <c r="Q10" s="6" t="inlineStr">
+      <c r="R15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Notizen</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
     </row>
     <row r="16">
       <c r="A16" s="7"/>
@@ -426,16 +370,17 @@
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="9"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="10"/>
       <c r="L16" s="9"/>
       <c r="M16" s="9"/>
       <c r="N16" s="9"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="7"/>
       <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
     </row>
     <row r="17">
       <c r="A17" s="7"/>
@@ -445,16 +390,17 @@
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="9"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="10"/>
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="9"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="7"/>
       <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
     </row>
     <row r="18">
       <c r="A18" s="7"/>
@@ -464,16 +410,17 @@
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="9"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="10"/>
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
       <c r="N18" s="9"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="9"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="7"/>
       <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
     </row>
     <row r="19">
       <c r="A19" s="7"/>
@@ -483,16 +430,17 @@
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="9"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="10"/>
       <c r="L19" s="9"/>
       <c r="M19" s="9"/>
       <c r="N19" s="9"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="7"/>
       <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
     </row>
     <row r="20">
       <c r="A20" s="7"/>
@@ -502,16 +450,17 @@
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="9"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="10"/>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="7"/>
       <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
     </row>
     <row r="21">
       <c r="A21" s="7"/>
@@ -521,16 +470,17 @@
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="9"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="10"/>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="7"/>
       <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
     </row>
     <row r="22">
       <c r="A22" s="7"/>
@@ -540,16 +490,17 @@
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="9"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="10"/>
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="7"/>
       <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
     </row>
     <row r="23">
       <c r="A23" s="7"/>
@@ -559,16 +510,17 @@
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="9"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="10"/>
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="9"/>
+      <c r="O23" s="9"/>
+      <c r="P23" s="7"/>
       <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
     </row>
     <row r="24">
       <c r="A24" s="7"/>
@@ -578,16 +530,17 @@
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="9"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="10"/>
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="9"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="7"/>
       <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
     </row>
     <row r="25">
       <c r="A25" s="7"/>
@@ -597,16 +550,17 @@
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="9"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="10"/>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
-      <c r="O25" s="7"/>
-      <c r="P25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="7"/>
       <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
     </row>
     <row r="26">
       <c r="A26" s="7"/>
@@ -616,16 +570,17 @@
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="9"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="10"/>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="9"/>
+      <c r="O26" s="9"/>
+      <c r="P26" s="7"/>
       <c r="Q26" s="9"/>
+      <c r="R26" s="9"/>
     </row>
     <row r="27">
       <c r="A27" s="7"/>
@@ -635,16 +590,17 @@
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="9"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="10"/>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="9"/>
+      <c r="O27" s="9"/>
+      <c r="P27" s="7"/>
       <c r="Q27" s="9"/>
+      <c r="R27" s="9"/>
     </row>
     <row r="28">
       <c r="A28" s="7"/>
@@ -654,16 +610,17 @@
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="9"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="10"/>
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="9"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="7"/>
       <c r="Q28" s="9"/>
+      <c r="R28" s="9"/>
     </row>
     <row r="29">
       <c r="A29" s="7"/>
@@ -673,16 +630,17 @@
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="9"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="10"/>
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="9"/>
+      <c r="O29" s="9"/>
+      <c r="P29" s="7"/>
       <c r="Q29" s="9"/>
+      <c r="R29" s="9"/>
     </row>
     <row r="30">
       <c r="A30" s="7"/>
@@ -692,16 +650,17 @@
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="9"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="10"/>
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="9"/>
+      <c r="O30" s="9"/>
+      <c r="P30" s="7"/>
       <c r="Q30" s="9"/>
+      <c r="R30" s="9"/>
     </row>
     <row r="31">
       <c r="A31" s="7"/>
@@ -711,16 +670,17 @@
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="9"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="10"/>
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="9"/>
+      <c r="O31" s="9"/>
+      <c r="P31" s="7"/>
       <c r="Q31" s="9"/>
+      <c r="R31" s="9"/>
     </row>
     <row r="32">
       <c r="A32" s="7"/>
@@ -730,16 +690,17 @@
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="9"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="10"/>
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="9"/>
+      <c r="O32" s="9"/>
+      <c r="P32" s="7"/>
       <c r="Q32" s="9"/>
+      <c r="R32" s="9"/>
     </row>
     <row r="33">
       <c r="A33" s="7"/>
@@ -749,16 +710,17 @@
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="9"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="10"/>
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="7"/>
       <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
     </row>
     <row r="34">
       <c r="A34" s="7"/>
@@ -768,16 +730,17 @@
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="9"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="10"/>
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="7"/>
       <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
     </row>
     <row r="35">
       <c r="A35" s="7"/>
@@ -787,35 +750,140 @@
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="9"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="10"/>
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
-      <c r="O35" s="7"/>
-      <c r="P35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="7"/>
       <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="7"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="9"/>
+      <c r="O37" s="9"/>
+      <c r="P37" s="7"/>
+      <c r="Q37" s="9"/>
+      <c r="R37" s="9"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
+      <c r="O38" s="9"/>
+      <c r="P38" s="7"/>
+      <c r="Q38" s="9"/>
+      <c r="R38" s="9"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="9"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="9"/>
+      <c r="M39" s="9"/>
+      <c r="N39" s="9"/>
+      <c r="O39" s="9"/>
+      <c r="P39" s="7"/>
+      <c r="Q39" s="9"/>
+      <c r="R39" s="9"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="7"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="9"/>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9"/>
+      <c r="O40" s="9"/>
+      <c r="P40" s="7"/>
+      <c r="Q40" s="9"/>
+      <c r="R40" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A2:Q2"/>
+  <mergeCells count="11">
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:R2"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:I12"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="B11:B310">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="C16:C315">
       <formula1>"Stiftung,Sparkasse,Volksbank / Bank,Unternehmen,Soziallotterie,Öffentliche Förderung,Kirchliche Stelle,Sonstiges"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="C11:C310">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="D16:D315">
       <formula1>"Portal,E-Mail,Brief,Persönlich,Telefon,Sonstiges"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="O11:O310">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="P16:P315">
       <formula1>"sehr wahrscheinlich,wahrscheinlich,unsicher,unwahrscheinlich,sehr unwahrscheinlich"</formula1>
     </dataValidation>
   </dataValidations>
@@ -839,299 +907,345 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="49" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diese Datei ist die Vorlage für den Förderplan eines Bedarfs aus der Bedarfsliste (Fundraising, Malteser Hilfsdienst e. V., Diözese Paderborn). Sie wird von Hand oder von einer KI ausgefüllt und danach in der Bedarfsliste über „Aus Excel übernehmen“ eingelesen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Auftrag: Finde Förderer, die zum Bedarf oben im Blatt „Förderplan“ passen – Stiftungen, Sparkassen und Volksbanken, Unternehmen, Soziallotterien, öffentliche und kirchliche Förderprogramme. Förderer mit Bezug zur Region der Gliederung zuerst. Prüfe Satzungszweck, Förderrichtlinien, Fristen und Förderhöhe auf den Seiten der Förderer und nenne die Quellen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Regeln</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t xml:space="preserve">Diese Datei ist die Vorlage für den Förderplan eines Bedarfs aus der Bedarfsliste (Fundraising, Malteser Hilfsdienst e. V., Diözese Paderborn). Sie wird von Hand oder von Copilot ausgefüllt und danach in der Bedarfsliste über „Excel übernehmen“ eingelesen. Der Bedarf mit Summe und noch offenem Betrag steht oben im Blatt „Förderplan“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auftrag</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Finde Förderer, die zu diesem Bedarf passen: Stiftungen, Sparkassen und Volksbanken, Unternehmen, Soziallotterien sowie öffentliche und kirchliche Förderprogramme. Förderer mit Bezug zum Erzbistum Paderborn und zu NRW zuerst, danach bundesweit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Je Förderer genau eine Zeile im Blatt „Förderplan“, ab der Zeile unter den Überschriften.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t xml:space="preserve">2. Prüfe jeden Förderer auf seinen eigenen Seiten: Satzungszweck, Förderrichtlinien, Antragsfristen, übliche Förderhöhe, geforderter Eigenanteil und Antragsweg. Nenne die Links als Quellen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Spaltenüberschriften, Blattnamen und die Angaben oben (Bedarf, Kennung) nicht ändern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Schon eingetragene Förderer ergänzen, nicht löschen oder doppelt anlegen.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">3. Förderer, die im Blatt „Förderplan“ schon stehen, nicht doppelt anlegen. Steht dort „zugesagt“ oder „abgelehnt“, die Zeile nicht ändern; sonst nur leere Zellen ergänzen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Datum immer als TT.MM.JJJJ, Beträge nur als Zahl in Euro (ohne Text).</t>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umfang</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">8 bis 12 Förderer, sortiert nach Erfolgsaussicht. Lieber weniger Förderer mit Beleg als viele unsichere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regeln</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Je Förderer genau eine Zeile im Blatt „Förderplan“, ab der Zeile unter den Überschriften.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Spaltenüberschriften, Blattnamen und die Angaben oben (Bedarf, Kennung) nicht ändern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Datum immer als TT.MM.JJJJ, Beträge nur als Zahl in Euro (ohne Text).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Art, Antragsweg und Einschätzung aus der Auswahlliste der Zelle wählen.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">• Unsicheres als solches kennzeichnen (z. B. „laut Website 2025, nicht bestätigt“). Nichts erfinden: lieber eine Zelle leer lassen.</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Spalte</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Was gehört hinein</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Förderer</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name der Stiftung, Bank, Firma oder des Förderprogramms – genau so, wie er in der Förder-Kartei steht, falls er dort schon vorkommt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Art</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aus der Auswahlliste. Auswahl: Stiftung · Sparkasse · Volksbank / Bank · Unternehmen · Soziallotterie · Öffentliche Förderung · Kirchliche Stelle · Sonstiges</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Antragsweg</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wie der Antrag gestellt wird – aus der Auswahlliste. Auswahl: Portal · E-Mail · Brief · Persönlich · Telefon · Sonstiges</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ansprechperson oder Portal</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name und Funktion der zuständigen Person oder Name des Antragsportals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E-Mail</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E-Mail-Adresse der Ansprechperson oder der Förderstelle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Telefon</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Telefonnummer.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Website oder Portal-Link</t>
+          <t xml:space="preserve">Förderer</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link zur Förderseite oder zum Antragsportal.</t>
+          <t xml:space="preserve">Name der Stiftung, Bank, Firma oder des Förderprogramms – genau so, wie er in der Förder-Kartei steht, falls er dort schon vorkommt.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antragsfrist</t>
+          <t xml:space="preserve">Stand in der Bedarfsliste</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nächster Einsendeschluss als Datum (TT.MM.JJJJ). Laufende Antragstellung: leer lassen und unter „Weitere Fristen und Termine“ notieren.</t>
+          <t xml:space="preserve">Nur zur Information: wie weit der Förderer schon ist. Wird nicht eingelesen. Bei neuen Förderern leer lassen.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weitere Fristen und Termine</t>
+          <t xml:space="preserve">Art</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vergabesitzungen, Stichtage, Bearbeitungszeit, „laufend“ usw.</t>
+          <t xml:space="preserve">Aus der Auswahlliste. Auswahl: Stiftung · Sparkasse · Volksbank / Bank · Unternehmen · Soziallotterie · Öffentliche Förderung · Kirchliche Stelle · Sonstiges</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erwartete Summe (€)</t>
+          <t xml:space="preserve">Antragsweg</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wie viel von diesem Förderer zu erwarten ist bzw. beantragt werden sollte – eine feste Summe, nur die Zahl in Euro.</t>
+          <t xml:space="preserve">Wie der Antrag gestellt wird – aus der Auswahlliste. Auswahl: Portal · E-Mail · Brief · Persönlich · Telefon · Sonstiges</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Übliche Fördersumme</t>
+          <t xml:space="preserve">Ansprechperson oder Portal</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Typische oder maximale Förderhöhe laut Richtlinien oder Förderhistorie.</t>
+          <t xml:space="preserve">Name und Funktion der zuständigen Person oder Name des Antragsportals.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eigenanteil gefordert</t>
+          <t xml:space="preserve">E-Mail</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ob und wie viel Eigenanteil verlangt wird.</t>
+          <t xml:space="preserve">E-Mail-Adresse der Ansprechperson oder der Förderstelle.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pro – warum passt das?</t>
+          <t xml:space="preserve">Telefon</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Begründung: Satzungszweck, Förderschwerpunkt, Regionalbezug, frühere Förderungen.</t>
+          <t xml:space="preserve">Telefonnummer.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contra – Knackpunkte</t>
+          <t xml:space="preserve">Website oder Portal-Link</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wo es haken kann und worauf der Antrag den Fokus legen sollte.</t>
+          <t xml:space="preserve">Link zur Förderseite oder zum Antragsportal.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Einschätzung</t>
+          <t xml:space="preserve">Antragsfrist</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wie wahrscheinlich eine Förderung ist – nur: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich. Auswahl: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich</t>
+          <t xml:space="preserve">Nächster Einsendeschluss als Datum (TT.MM.JJJJ). Laufende Antragstellung: leer lassen und unter „Weitere Fristen und Termine“ notieren.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quellen</t>
+          <t xml:space="preserve">Weitere Fristen und Termine</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Links zu Satzung, Förderrichtlinien und weiteren Belegen.</t>
+          <t xml:space="preserve">Vergabesitzungen, Stichtage, Bearbeitungszeit, „laufend“ usw.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Erwartete Summe (€)</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie viel von diesem Förderer zu erwarten ist bzw. beantragt werden sollte – eine feste Summe, nur die Zahl in Euro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Übliche Fördersumme</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Typische oder maximale Förderhöhe laut Richtlinien oder Förderhistorie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eigenanteil gefordert</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ob und wie viel Eigenanteil verlangt wird.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pro – warum passt das?</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Begründung: Satzungszweck, Förderschwerpunkt, Regionalbezug, frühere Förderungen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contra – Knackpunkte</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wo es haken kann und worauf der Antrag den Fokus legen sollte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Einschätzung</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie wahrscheinlich eine Förderung ist – nur: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich. Auswahl: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quellen</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Links zu Satzung, Förderrichtlinien und weiteren Belegen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
           <t xml:space="preserve">Notizen</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Alles Weitere.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="14">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Bedarfsliste 0.16: Korrekturen zur Förderrecherche
- Recherche-Excel mit Titel, Gliederung und Kürzel der Kennung; Suche über das Kürzel, neueste passende Datei (auch Kopien)
- Unveränderte Excel: Hinweis mit Gründen und „Andere Datei wählen …“
- Prompt: Excel anhängen, Websuche Pflicht (sonst Abbruch), nur geöffnete Links als Quelle
- Umfang nach offenem Betrag gestaffelt, keine Zielsumme
- Kartei-Blatt ohne Notizen, Hinweis im Dialog, was an Copilot geht
- Pfad: Anführungszeichen aus „Als Pfad kopieren“ entfernen
- README: Regeln für die geplanten Hinweise aus dem Postfach

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="34" customHeight="1">
+    <row r="6" ht="49" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. Prüfe jeden Förderer auf seinen eigenen Seiten: Satzungszweck, Förderrichtlinien, Antragsfristen, übliche Förderhöhe, geforderter Eigenanteil und Antragsweg. Nenne die Links als Quellen.</t>
+          <t xml:space="preserve">2. Recherchiere im Web und prüfe jeden Förderer auf seinen eigenen Seiten: Satzungszweck, Förderrichtlinien, Antragsfristen, übliche Förderhöhe, geforderter Eigenanteil und Antragsweg. Trage als Quellen nur Links ein, die du dabei tatsächlich geöffnet hast. Wenn du nicht im Web suchen kannst, brich ab und sag es mir.</t>
         </is>
       </c>
     </row>
@@ -951,10 +951,10 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="49" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 bis 12 Förderer, sortiert nach Erfolgsaussicht. Lieber weniger Förderer mit Beleg als viele unsichere.</t>
+          <t xml:space="preserve">5 bis 8 Förderer, sortiert nach Erfolgsaussicht. Die erwartete Summe je Förderer realistisch aus Förderhistorie, Richtlinien oder üblicher Förderhöhe ableiten; geht das nicht, die Zelle leer lassen. Nicht auf eine Gesamtsumme hinrechnen. Lieber weniger Förderer mit Beleg als viele unsichere.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bedarfsliste 0.17: Liste dauerhaft bearbeitbar, Zeitstrahl, Details als Fenster
- Liste: Bearbeiten ohne Strg, Strg + Klick öffnet den Bedarf; ganze Zeile beim Überfahren hervorgehoben
- „+ Bedarf“ legt die Zeile in der Liste an (Name → Summe → Ort → Ansprechperson → Deadline mit Enter)
- Verwendungsnachweis standardmäßig nötig (gespeicherte Daten einmalig umgestellt)
- Zeitstrahl zur Frist des Verwendungsnachweises: grau, gelb ab 30 Tagen, rot ab 7 Tagen
- Förderer ohne Stand „in Vorbereitung“
- Kreisdiagramm mit allen Beschriftungen beim Überfahren, Summe oben größer
- Kontakt und Details als Fenster mit Knöpfen für E-Mail, Telefon, Website; Quellen als Links
- Pro/Contra drei Zeilen mit mehr Abstand; Prompt: Quellen je Zeile, kurze Felder

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -997,241 +997,255 @@
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• Kurze Felder kurz halten: „Ansprechperson oder Portal“, „Übliche Fördersumme“ und „Eigenanteil gefordert“ höchstens etwa 80 Zeichen – Erläuterungen gehören in „Notizen“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Quellen: je Link eine eigene Zeile in der Zelle, nur die Adresse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Unsicheres als solches kennzeichnen (z. B. „laut Website 2025, nicht bestätigt“). Nichts erfinden: lieber eine Zelle leer lassen.</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Spalte</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Was gehört hinein</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Förderer</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name der Stiftung, Bank, Firma oder des Förderprogramms – genau so, wie er in der Förder-Kartei steht, falls er dort schon vorkommt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stand in der Bedarfsliste</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nur zur Information: wie weit der Förderer schon ist. Wird nicht eingelesen. Bei neuen Förderern leer lassen.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Art</t>
+          <t xml:space="preserve">Förderer</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aus der Auswahlliste. Auswahl: Stiftung · Sparkasse · Volksbank / Bank · Unternehmen · Soziallotterie · Öffentliche Förderung · Kirchliche Stelle · Sonstiges</t>
+          <t xml:space="preserve">Name der Stiftung, Bank, Firma oder des Förderprogramms – genau so, wie er in der Förder-Kartei steht, falls er dort schon vorkommt.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antragsweg</t>
+          <t xml:space="preserve">Stand in der Bedarfsliste</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wie der Antrag gestellt wird – aus der Auswahlliste. Auswahl: Portal · E-Mail · Brief · Persönlich · Telefon · Sonstiges</t>
+          <t xml:space="preserve">Nur zur Information: wie weit der Förderer schon ist. Wird nicht eingelesen. Bei neuen Förderern leer lassen.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ansprechperson oder Portal</t>
+          <t xml:space="preserve">Art</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name und Funktion der zuständigen Person oder Name des Antragsportals.</t>
+          <t xml:space="preserve">Aus der Auswahlliste. Auswahl: Stiftung · Sparkasse · Volksbank / Bank · Unternehmen · Soziallotterie · Öffentliche Förderung · Kirchliche Stelle · Sonstiges</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">E-Mail</t>
+          <t xml:space="preserve">Antragsweg</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">E-Mail-Adresse der Ansprechperson oder der Förderstelle.</t>
+          <t xml:space="preserve">Wie der Antrag gestellt wird – aus der Auswahlliste. Auswahl: Portal · E-Mail · Brief · Persönlich · Telefon · Sonstiges</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telefon</t>
+          <t xml:space="preserve">Ansprechperson oder Portal</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telefonnummer.</t>
+          <t xml:space="preserve">Name und Funktion der zuständigen Person oder Name des Antragsportals – kurz, höchstens etwa 80 Zeichen.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Website oder Portal-Link</t>
+          <t xml:space="preserve">E-Mail</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link zur Förderseite oder zum Antragsportal.</t>
+          <t xml:space="preserve">E-Mail-Adresse der Ansprechperson oder der Förderstelle.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antragsfrist</t>
+          <t xml:space="preserve">Telefon</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nächster Einsendeschluss als Datum (TT.MM.JJJJ). Laufende Antragstellung: leer lassen und unter „Weitere Fristen und Termine“ notieren.</t>
+          <t xml:space="preserve">Telefonnummer.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weitere Fristen und Termine</t>
+          <t xml:space="preserve">Website oder Portal-Link</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vergabesitzungen, Stichtage, Bearbeitungszeit, „laufend“ usw.</t>
+          <t xml:space="preserve">Link zur Förderseite oder zum Antragsportal.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erwartete Summe (€)</t>
+          <t xml:space="preserve">Antragsfrist</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wie viel von diesem Förderer zu erwarten ist bzw. beantragt werden sollte – eine feste Summe, nur die Zahl in Euro.</t>
+          <t xml:space="preserve">Nächster Einsendeschluss als Datum (TT.MM.JJJJ). Laufende Antragstellung: leer lassen und unter „Weitere Fristen und Termine“ notieren.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Übliche Fördersumme</t>
+          <t xml:space="preserve">Weitere Fristen und Termine</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Typische oder maximale Förderhöhe laut Richtlinien oder Förderhistorie.</t>
+          <t xml:space="preserve">Vergabesitzungen, Stichtage, Bearbeitungszeit, „laufend“ usw.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eigenanteil gefordert</t>
+          <t xml:space="preserve">Erwartete Summe (€)</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ob und wie viel Eigenanteil verlangt wird.</t>
+          <t xml:space="preserve">Wie viel von diesem Förderer zu erwarten ist bzw. beantragt werden sollte – eine feste Summe, nur die Zahl in Euro.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pro – warum passt das?</t>
+          <t xml:space="preserve">Übliche Fördersumme</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Begründung: Satzungszweck, Förderschwerpunkt, Regionalbezug, frühere Förderungen.</t>
+          <t xml:space="preserve">Typische oder maximale Förderhöhe laut Richtlinien oder Förderhistorie – kurz, z. B. „1.000–5.000 €, max. 10.000 €“ (höchstens etwa 80 Zeichen; Erläuterungen in „Notizen“).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contra – Knackpunkte</t>
+          <t xml:space="preserve">Eigenanteil gefordert</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wo es haken kann und worauf der Antrag den Fokus legen sollte.</t>
+          <t xml:space="preserve">Ob und wie viel Eigenanteil verlangt wird – kurz, z. B. „ja, mind. 20 %“ oder „nein“ (höchstens etwa 80 Zeichen; Erläuterungen in „Notizen“).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Einschätzung</t>
+          <t xml:space="preserve">Pro – warum passt das?</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wie wahrscheinlich eine Förderung ist – nur: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich. Auswahl: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich</t>
+          <t xml:space="preserve">Begründung: Satzungszweck, Förderschwerpunkt, Regionalbezug, frühere Förderungen.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quellen</t>
+          <t xml:space="preserve">Contra – Knackpunkte</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Links zu Satzung, Förderrichtlinien und weiteren Belegen.</t>
+          <t xml:space="preserve">Wo es haken kann und worauf der Antrag den Fokus legen sollte.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Einschätzung</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie wahrscheinlich eine Förderung ist – nur: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich. Auswahl: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quellen</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Links zu Satzung, Förderrichtlinien und weiteren Belegen – je Link eine eigene Zeile in der Zelle (Zeilenumbruch), nur die Adresse, keine Trennzeichen wie „;“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
           <t xml:space="preserve">Notizen</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Alles Weitere.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
@@ -1246,6 +1260,8 @@
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Bedarfsliste 0.21: Förderer-Fenster mit Summe, Wahrscheinlichkeit und bis zu drei Kontakten
- Kopf: Summe neben dem Namen, Wahrscheinlichkeit rechts, beides änderbar; ohne Stand und „Antrag stellt“
- Kontakte als Liste mit Hauptkontakt (Stern), Links und Knöpfen; Stift zum Bearbeiten, höchstens drei; Kartei-Kontakte mit Vermerk
- Rechts ohne Überschrift; feste Höhe für drei Kontakte, lange Texte scrollen im eigenen Bereich
- Daten: bisherige Ansprechperson/E-Mail/Telefon werden zum ersten Kontakt; Excel-Spalte „Kontakte“ je Person eine Zeile

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -127,11 +127,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -158,7 +158,7 @@
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="32" customWidth="1"/>
@@ -293,7 +293,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ansprechperson oder Portal</t>
+          <t xml:space="preserve">Kontakte</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -367,500 +367,500 @@
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
+      <c r="E16" s="8"/>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="8"/>
       <c r="K16" s="10"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
       <c r="P16" s="7"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
     </row>
     <row r="17">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
+      <c r="E17" s="8"/>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="8"/>
       <c r="K17" s="10"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
       <c r="P17" s="7"/>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="9"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
     </row>
     <row r="18">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="8"/>
       <c r="K18" s="10"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
       <c r="P18" s="7"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="9"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
     </row>
     <row r="19">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="8"/>
       <c r="K19" s="10"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
       <c r="P19" s="7"/>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="9"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
     </row>
     <row r="20">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="8"/>
       <c r="K20" s="10"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
       <c r="P20" s="7"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="9"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
     </row>
     <row r="21">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="8"/>
       <c r="K21" s="10"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
       <c r="P21" s="7"/>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="9"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="8"/>
     </row>
     <row r="22">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="8"/>
       <c r="K22" s="10"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
       <c r="P22" s="7"/>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="9"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
     </row>
     <row r="23">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
+      <c r="E23" s="8"/>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="8"/>
       <c r="K23" s="10"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
       <c r="P23" s="7"/>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="8"/>
     </row>
     <row r="24">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
+      <c r="E24" s="8"/>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="8"/>
       <c r="K24" s="10"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
+      <c r="L24" s="8"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
       <c r="P24" s="7"/>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="9"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="8"/>
     </row>
     <row r="25">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="8"/>
       <c r="K25" s="10"/>
-      <c r="L25" s="9"/>
-      <c r="M25" s="9"/>
-      <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
       <c r="P25" s="7"/>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="9"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
     </row>
     <row r="26">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="8"/>
       <c r="K26" s="10"/>
-      <c r="L26" s="9"/>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
       <c r="P26" s="7"/>
-      <c r="Q26" s="9"/>
-      <c r="R26" s="9"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="8"/>
     </row>
     <row r="27">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
+      <c r="E27" s="8"/>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="8"/>
       <c r="K27" s="10"/>
-      <c r="L27" s="9"/>
-      <c r="M27" s="9"/>
-      <c r="N27" s="9"/>
-      <c r="O27" s="9"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
       <c r="P27" s="7"/>
-      <c r="Q27" s="9"/>
-      <c r="R27" s="9"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="8"/>
     </row>
     <row r="28">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="8"/>
       <c r="K28" s="10"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
       <c r="P28" s="7"/>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="9"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="8"/>
     </row>
     <row r="29">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
+      <c r="E29" s="8"/>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="8"/>
       <c r="K29" s="10"/>
-      <c r="L29" s="9"/>
-      <c r="M29" s="9"/>
-      <c r="N29" s="9"/>
-      <c r="O29" s="9"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
       <c r="P29" s="7"/>
-      <c r="Q29" s="9"/>
-      <c r="R29" s="9"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
     </row>
     <row r="30">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
+      <c r="E30" s="8"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="8"/>
       <c r="K30" s="10"/>
-      <c r="L30" s="9"/>
-      <c r="M30" s="9"/>
-      <c r="N30" s="9"/>
-      <c r="O30" s="9"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
       <c r="P30" s="7"/>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="9"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
     </row>
     <row r="31">
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
+      <c r="E31" s="8"/>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="8"/>
       <c r="K31" s="10"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
-      <c r="N31" s="9"/>
-      <c r="O31" s="9"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
       <c r="P31" s="7"/>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="9"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
     </row>
     <row r="32">
       <c r="A32" s="7"/>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
+      <c r="E32" s="8"/>
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="9"/>
+      <c r="I32" s="9"/>
+      <c r="J32" s="8"/>
       <c r="K32" s="10"/>
-      <c r="L32" s="9"/>
-      <c r="M32" s="9"/>
-      <c r="N32" s="9"/>
-      <c r="O32" s="9"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
       <c r="P32" s="7"/>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="9"/>
+      <c r="Q32" s="8"/>
+      <c r="R32" s="8"/>
     </row>
     <row r="33">
       <c r="A33" s="7"/>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
+      <c r="E33" s="8"/>
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="8"/>
       <c r="K33" s="10"/>
-      <c r="L33" s="9"/>
-      <c r="M33" s="9"/>
-      <c r="N33" s="9"/>
-      <c r="O33" s="9"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="8"/>
       <c r="P33" s="7"/>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="9"/>
+      <c r="Q33" s="8"/>
+      <c r="R33" s="8"/>
     </row>
     <row r="34">
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
+      <c r="E34" s="8"/>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="8"/>
       <c r="K34" s="10"/>
-      <c r="L34" s="9"/>
-      <c r="M34" s="9"/>
-      <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
       <c r="P34" s="7"/>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="9"/>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
     </row>
     <row r="35">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
+      <c r="E35" s="8"/>
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="8"/>
       <c r="K35" s="10"/>
-      <c r="L35" s="9"/>
-      <c r="M35" s="9"/>
-      <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
       <c r="P35" s="7"/>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
     </row>
     <row r="36">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
+      <c r="E36" s="8"/>
       <c r="F36" s="7"/>
       <c r="G36" s="7"/>
       <c r="H36" s="7"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="8"/>
       <c r="K36" s="10"/>
-      <c r="L36" s="9"/>
-      <c r="M36" s="9"/>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
       <c r="P36" s="7"/>
-      <c r="Q36" s="9"/>
-      <c r="R36" s="9"/>
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
     </row>
     <row r="37">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
+      <c r="E37" s="8"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="9"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="8"/>
       <c r="K37" s="10"/>
-      <c r="L37" s="9"/>
-      <c r="M37" s="9"/>
-      <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
       <c r="P37" s="7"/>
-      <c r="Q37" s="9"/>
-      <c r="R37" s="9"/>
+      <c r="Q37" s="8"/>
+      <c r="R37" s="8"/>
     </row>
     <row r="38">
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
+      <c r="E38" s="8"/>
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="8"/>
       <c r="K38" s="10"/>
-      <c r="L38" s="9"/>
-      <c r="M38" s="9"/>
-      <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
       <c r="P38" s="7"/>
-      <c r="Q38" s="9"/>
-      <c r="R38" s="9"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
     </row>
     <row r="39">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
+      <c r="E39" s="8"/>
       <c r="F39" s="7"/>
       <c r="G39" s="7"/>
       <c r="H39" s="7"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="9"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="8"/>
       <c r="K39" s="10"/>
-      <c r="L39" s="9"/>
-      <c r="M39" s="9"/>
-      <c r="N39" s="9"/>
-      <c r="O39" s="9"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
       <c r="P39" s="7"/>
-      <c r="Q39" s="9"/>
-      <c r="R39" s="9"/>
+      <c r="Q39" s="8"/>
+      <c r="R39" s="8"/>
     </row>
     <row r="40">
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
+      <c r="E40" s="8"/>
       <c r="F40" s="7"/>
       <c r="G40" s="7"/>
       <c r="H40" s="7"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="8"/>
       <c r="K40" s="10"/>
-      <c r="L40" s="9"/>
-      <c r="M40" s="9"/>
-      <c r="N40" s="9"/>
-      <c r="O40" s="9"/>
+      <c r="L40" s="8"/>
+      <c r="M40" s="8"/>
+      <c r="N40" s="8"/>
+      <c r="O40" s="8"/>
       <c r="P40" s="7"/>
-      <c r="Q40" s="9"/>
-      <c r="R40" s="9"/>
+      <c r="Q40" s="8"/>
+      <c r="R40" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -994,258 +994,265 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="34" customHeight="1">
+    <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Kurze Felder kurz halten: „Ansprechperson oder Portal“, „Übliche Fördersumme“ und „Eigenanteil gefordert“ höchstens etwa 80 Zeichen – Erläuterungen gehören in „Notizen“.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t xml:space="preserve">• Kontakte: bis zu drei Personen, je Person eine Zeile in der Zelle „Name; Funktion; E-Mail; Telefon“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• Kurze Felder kurz halten: „Übliche Fördersumme“ und „Eigenanteil gefordert“ höchstens etwa 80 Zeichen – Erläuterungen gehören in „Notizen“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Quellen: je Link eine eigene Zeile in der Zelle, nur die Adresse.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">• Unsicheres als solches kennzeichnen (z. B. „laut Website 2025, nicht bestätigt“). Nichts erfinden: lieber eine Zelle leer lassen.</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Spalte</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Was gehört hinein</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Förderer</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name der Stiftung, Bank, Firma oder des Förderprogramms – genau so, wie er in der Förder-Kartei steht, falls er dort schon vorkommt.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stand in der Bedarfsliste</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nur zur Information: wie weit der Förderer schon ist. Wird nicht eingelesen. Bei neuen Förderern leer lassen.</t>
+          <t xml:space="preserve">Förderer</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name der Stiftung, Bank, Firma oder des Förderprogramms – genau so, wie er in der Förder-Kartei steht, falls er dort schon vorkommt.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Art</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aus der Auswahlliste. Auswahl: Stiftung · Sparkasse · Volksbank / Bank · Unternehmen · Soziallotterie · Öffentliche Förderung · Kirchliche Stelle · Sonstiges</t>
+          <t xml:space="preserve">Stand in der Bedarfsliste</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nur zur Information: wie weit der Förderer schon ist. Wird nicht eingelesen. Bei neuen Förderern leer lassen.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antragsweg</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wie der Antrag gestellt wird – aus der Auswahlliste. Auswahl: Portal · E-Mail · Brief · Persönlich · Telefon · Sonstiges</t>
+          <t xml:space="preserve">Art</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aus der Auswahlliste. Auswahl: Stiftung · Sparkasse · Volksbank / Bank · Unternehmen · Soziallotterie · Öffentliche Förderung · Kirchliche Stelle · Sonstiges</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ansprechperson oder Portal</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name und Funktion der zuständigen Person oder Name des Antragsportals – kurz, höchstens etwa 80 Zeichen.</t>
+          <t xml:space="preserve">Antragsweg</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie der Antrag gestellt wird – aus der Auswahlliste. Auswahl: Portal · E-Mail · Brief · Persönlich · Telefon · Sonstiges</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">E-Mail</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E-Mail-Adresse der Ansprechperson oder der Förderstelle.</t>
+          <t xml:space="preserve">Kontakte</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bis zu drei Ansprechpersonen, je Person eine Zeile in der Zelle: Name; Funktion; E-Mail; Telefon (Unbekanntes weglassen). Wichtigste Person zuerst. Bei Antrag nur über ein Portal: Name des Portals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telefon</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Telefonnummer.</t>
+          <t xml:space="preserve">E-Mail</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Allgemeine E-Mail-Adresse der Förderstelle (gilt für die erste Person, wenn sie keine eigene hat).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Website oder Portal-Link</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Link zur Förderseite oder zum Antragsportal.</t>
+          <t xml:space="preserve">Telefon</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Allgemeine Telefonnummer der Förderstelle (gilt für die erste Person, wenn sie keine eigene hat).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antragsfrist</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nächster Einsendeschluss als Datum (TT.MM.JJJJ). Laufende Antragstellung: leer lassen und unter „Weitere Fristen und Termine“ notieren.</t>
+          <t xml:space="preserve">Website oder Portal-Link</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Link zur Förderseite oder zum Antragsportal.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weitere Fristen und Termine</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vergabesitzungen, Stichtage, Bearbeitungszeit, „laufend“ usw.</t>
+          <t xml:space="preserve">Antragsfrist</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nächster Einsendeschluss als Datum (TT.MM.JJJJ). Laufende Antragstellung: leer lassen und unter „Weitere Fristen und Termine“ notieren.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erwartete Summe (€)</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wie viel von diesem Förderer zu erwarten ist bzw. beantragt werden sollte – eine feste Summe, nur die Zahl in Euro.</t>
+          <t xml:space="preserve">Weitere Fristen und Termine</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vergabesitzungen, Stichtage, Bearbeitungszeit, „laufend“ usw.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Übliche Fördersumme</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Typische oder maximale Förderhöhe laut Richtlinien oder Förderhistorie – kurz, z. B. „1.000–5.000 €, max. 10.000 €“ (höchstens etwa 80 Zeichen; Erläuterungen in „Notizen“).</t>
+          <t xml:space="preserve">Erwartete Summe (€)</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie viel von diesem Förderer zu erwarten ist bzw. beantragt werden sollte – eine feste Summe, nur die Zahl in Euro.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eigenanteil gefordert</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ob und wie viel Eigenanteil verlangt wird – kurz, z. B. „ja, mind. 20 %“ oder „nein“ (höchstens etwa 80 Zeichen; Erläuterungen in „Notizen“).</t>
+          <t xml:space="preserve">Übliche Fördersumme</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Typische oder maximale Förderhöhe laut Richtlinien oder Förderhistorie – kurz, z. B. „1.000–5.000 €, max. 10.000 €“ (höchstens etwa 80 Zeichen; Erläuterungen in „Notizen“).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pro – warum passt das?</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Begründung: Satzungszweck, Förderschwerpunkt, Regionalbezug, frühere Förderungen.</t>
+          <t xml:space="preserve">Eigenanteil gefordert</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ob und wie viel Eigenanteil verlangt wird – kurz, z. B. „ja, mind. 20 %“ oder „nein“ (höchstens etwa 80 Zeichen; Erläuterungen in „Notizen“).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contra – Knackpunkte</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wo es haken kann und worauf der Antrag den Fokus legen sollte.</t>
+          <t xml:space="preserve">Pro – warum passt das?</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Begründung: Satzungszweck, Förderschwerpunkt, Regionalbezug, frühere Förderungen.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Einschätzung</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wie wahrscheinlich eine Förderung ist – nur: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich. Auswahl: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich</t>
+          <t xml:space="preserve">Contra – Knackpunkte</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wo es haken kann und worauf der Antrag den Fokus legen sollte.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quellen</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Links zu Satzung, Förderrichtlinien und weiteren Belegen – je Link eine eigene Zeile in der Zelle (Zeilenumbruch), nur die Adresse, keine Trennzeichen wie „;“.</t>
+          <t xml:space="preserve">Einschätzung</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie wahrscheinlich eine Förderung ist – nur: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich. Auswahl: sehr wahrscheinlich · wahrscheinlich · unsicher · unwahrscheinlich · sehr unwahrscheinlich</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Quellen</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Links zu Satzung, Förderrichtlinien und weiteren Belegen – je Link eine eigene Zeile in der Zelle (Zeilenumbruch), nur die Adresse, keine Trennzeichen wie „;“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
           <t xml:space="preserve">Notizen</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Alles Weitere.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
@@ -1262,6 +1269,7 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Bedarfsliste 0.37: Excel-Übernahme robust (Block 4 der Prüfung)
- readFoerderplan: Kopfzeile flexibel, nie Anleitung/Kartei/ausgeblendete Blätter, mehrere Blätter zusammengeführt, Platzhalter und Summenzeilen übergangen
- _Stand (ausgeblendet) in der Vorlage: Überschreiben nur geänderter Felder; zugesagte/abgelehnte Förderer nur ergänzen
- Telefon: Text-Format (numFmt 49) in Vorlagen, telText ergänzt führende 0; mailText, ohnePlatzhalter
- Personen: Namensvarianten, Meldung ohne Spalten, Ergänzen einmal je Fassung (z.pxl)
- kkey toleranter; Kartei: Gliederung-Varianten, Meldung, Konfliktkopie nachrangig, Links
- xlsxBook: _xHHHH_, <t/>, x:-Präfix, hidden, Hyperlinks, HYPERLINK-Formeln, t=d, date1904; Schreiben: ungültige Zeichen, 32767, NaN, hidden
- Tests: t11 (13 Prüfungen), t03/t04 angepasst

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -129,6 +129,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -369,11 +372,11 @@
       <c r="D16" s="7"/>
       <c r="E16" s="8"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="G16" s="9"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="9"/>
+      <c r="I16" s="10"/>
       <c r="J16" s="8"/>
-      <c r="K16" s="10"/>
+      <c r="K16" s="11"/>
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
@@ -389,11 +392,11 @@
       <c r="D17" s="7"/>
       <c r="E17" s="8"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="G17" s="9"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="9"/>
+      <c r="I17" s="10"/>
       <c r="J17" s="8"/>
-      <c r="K17" s="10"/>
+      <c r="K17" s="11"/>
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
@@ -409,11 +412,11 @@
       <c r="D18" s="7"/>
       <c r="E18" s="8"/>
       <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="G18" s="9"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="9"/>
+      <c r="I18" s="10"/>
       <c r="J18" s="8"/>
-      <c r="K18" s="10"/>
+      <c r="K18" s="11"/>
       <c r="L18" s="8"/>
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
@@ -429,11 +432,11 @@
       <c r="D19" s="7"/>
       <c r="E19" s="8"/>
       <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
+      <c r="G19" s="9"/>
       <c r="H19" s="7"/>
-      <c r="I19" s="9"/>
+      <c r="I19" s="10"/>
       <c r="J19" s="8"/>
-      <c r="K19" s="10"/>
+      <c r="K19" s="11"/>
       <c r="L19" s="8"/>
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
@@ -449,11 +452,11 @@
       <c r="D20" s="7"/>
       <c r="E20" s="8"/>
       <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="G20" s="9"/>
       <c r="H20" s="7"/>
-      <c r="I20" s="9"/>
+      <c r="I20" s="10"/>
       <c r="J20" s="8"/>
-      <c r="K20" s="10"/>
+      <c r="K20" s="11"/>
       <c r="L20" s="8"/>
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
@@ -469,11 +472,11 @@
       <c r="D21" s="7"/>
       <c r="E21" s="8"/>
       <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="G21" s="9"/>
       <c r="H21" s="7"/>
-      <c r="I21" s="9"/>
+      <c r="I21" s="10"/>
       <c r="J21" s="8"/>
-      <c r="K21" s="10"/>
+      <c r="K21" s="11"/>
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
@@ -489,11 +492,11 @@
       <c r="D22" s="7"/>
       <c r="E22" s="8"/>
       <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
+      <c r="G22" s="9"/>
       <c r="H22" s="7"/>
-      <c r="I22" s="9"/>
+      <c r="I22" s="10"/>
       <c r="J22" s="8"/>
-      <c r="K22" s="10"/>
+      <c r="K22" s="11"/>
       <c r="L22" s="8"/>
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
@@ -509,11 +512,11 @@
       <c r="D23" s="7"/>
       <c r="E23" s="8"/>
       <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
+      <c r="G23" s="9"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="9"/>
+      <c r="I23" s="10"/>
       <c r="J23" s="8"/>
-      <c r="K23" s="10"/>
+      <c r="K23" s="11"/>
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
@@ -529,11 +532,11 @@
       <c r="D24" s="7"/>
       <c r="E24" s="8"/>
       <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
+      <c r="G24" s="9"/>
       <c r="H24" s="7"/>
-      <c r="I24" s="9"/>
+      <c r="I24" s="10"/>
       <c r="J24" s="8"/>
-      <c r="K24" s="10"/>
+      <c r="K24" s="11"/>
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
@@ -549,11 +552,11 @@
       <c r="D25" s="7"/>
       <c r="E25" s="8"/>
       <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
+      <c r="G25" s="9"/>
       <c r="H25" s="7"/>
-      <c r="I25" s="9"/>
+      <c r="I25" s="10"/>
       <c r="J25" s="8"/>
-      <c r="K25" s="10"/>
+      <c r="K25" s="11"/>
       <c r="L25" s="8"/>
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>
@@ -569,11 +572,11 @@
       <c r="D26" s="7"/>
       <c r="E26" s="8"/>
       <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
+      <c r="G26" s="9"/>
       <c r="H26" s="7"/>
-      <c r="I26" s="9"/>
+      <c r="I26" s="10"/>
       <c r="J26" s="8"/>
-      <c r="K26" s="10"/>
+      <c r="K26" s="11"/>
       <c r="L26" s="8"/>
       <c r="M26" s="8"/>
       <c r="N26" s="8"/>
@@ -589,11 +592,11 @@
       <c r="D27" s="7"/>
       <c r="E27" s="8"/>
       <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
+      <c r="G27" s="9"/>
       <c r="H27" s="7"/>
-      <c r="I27" s="9"/>
+      <c r="I27" s="10"/>
       <c r="J27" s="8"/>
-      <c r="K27" s="10"/>
+      <c r="K27" s="11"/>
       <c r="L27" s="8"/>
       <c r="M27" s="8"/>
       <c r="N27" s="8"/>
@@ -609,11 +612,11 @@
       <c r="D28" s="7"/>
       <c r="E28" s="8"/>
       <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
+      <c r="G28" s="9"/>
       <c r="H28" s="7"/>
-      <c r="I28" s="9"/>
+      <c r="I28" s="10"/>
       <c r="J28" s="8"/>
-      <c r="K28" s="10"/>
+      <c r="K28" s="11"/>
       <c r="L28" s="8"/>
       <c r="M28" s="8"/>
       <c r="N28" s="8"/>
@@ -629,11 +632,11 @@
       <c r="D29" s="7"/>
       <c r="E29" s="8"/>
       <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
+      <c r="G29" s="9"/>
       <c r="H29" s="7"/>
-      <c r="I29" s="9"/>
+      <c r="I29" s="10"/>
       <c r="J29" s="8"/>
-      <c r="K29" s="10"/>
+      <c r="K29" s="11"/>
       <c r="L29" s="8"/>
       <c r="M29" s="8"/>
       <c r="N29" s="8"/>
@@ -649,11 +652,11 @@
       <c r="D30" s="7"/>
       <c r="E30" s="8"/>
       <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
+      <c r="G30" s="9"/>
       <c r="H30" s="7"/>
-      <c r="I30" s="9"/>
+      <c r="I30" s="10"/>
       <c r="J30" s="8"/>
-      <c r="K30" s="10"/>
+      <c r="K30" s="11"/>
       <c r="L30" s="8"/>
       <c r="M30" s="8"/>
       <c r="N30" s="8"/>
@@ -669,11 +672,11 @@
       <c r="D31" s="7"/>
       <c r="E31" s="8"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
+      <c r="G31" s="9"/>
       <c r="H31" s="7"/>
-      <c r="I31" s="9"/>
+      <c r="I31" s="10"/>
       <c r="J31" s="8"/>
-      <c r="K31" s="10"/>
+      <c r="K31" s="11"/>
       <c r="L31" s="8"/>
       <c r="M31" s="8"/>
       <c r="N31" s="8"/>
@@ -689,11 +692,11 @@
       <c r="D32" s="7"/>
       <c r="E32" s="8"/>
       <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
+      <c r="G32" s="9"/>
       <c r="H32" s="7"/>
-      <c r="I32" s="9"/>
+      <c r="I32" s="10"/>
       <c r="J32" s="8"/>
-      <c r="K32" s="10"/>
+      <c r="K32" s="11"/>
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
       <c r="N32" s="8"/>
@@ -709,11 +712,11 @@
       <c r="D33" s="7"/>
       <c r="E33" s="8"/>
       <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="G33" s="9"/>
       <c r="H33" s="7"/>
-      <c r="I33" s="9"/>
+      <c r="I33" s="10"/>
       <c r="J33" s="8"/>
-      <c r="K33" s="10"/>
+      <c r="K33" s="11"/>
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
       <c r="N33" s="8"/>
@@ -729,11 +732,11 @@
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
       <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="G34" s="9"/>
       <c r="H34" s="7"/>
-      <c r="I34" s="9"/>
+      <c r="I34" s="10"/>
       <c r="J34" s="8"/>
-      <c r="K34" s="10"/>
+      <c r="K34" s="11"/>
       <c r="L34" s="8"/>
       <c r="M34" s="8"/>
       <c r="N34" s="8"/>
@@ -749,11 +752,11 @@
       <c r="D35" s="7"/>
       <c r="E35" s="8"/>
       <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="G35" s="9"/>
       <c r="H35" s="7"/>
-      <c r="I35" s="9"/>
+      <c r="I35" s="10"/>
       <c r="J35" s="8"/>
-      <c r="K35" s="10"/>
+      <c r="K35" s="11"/>
       <c r="L35" s="8"/>
       <c r="M35" s="8"/>
       <c r="N35" s="8"/>
@@ -769,11 +772,11 @@
       <c r="D36" s="7"/>
       <c r="E36" s="8"/>
       <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
+      <c r="G36" s="9"/>
       <c r="H36" s="7"/>
-      <c r="I36" s="9"/>
+      <c r="I36" s="10"/>
       <c r="J36" s="8"/>
-      <c r="K36" s="10"/>
+      <c r="K36" s="11"/>
       <c r="L36" s="8"/>
       <c r="M36" s="8"/>
       <c r="N36" s="8"/>
@@ -789,11 +792,11 @@
       <c r="D37" s="7"/>
       <c r="E37" s="8"/>
       <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
+      <c r="G37" s="9"/>
       <c r="H37" s="7"/>
-      <c r="I37" s="9"/>
+      <c r="I37" s="10"/>
       <c r="J37" s="8"/>
-      <c r="K37" s="10"/>
+      <c r="K37" s="11"/>
       <c r="L37" s="8"/>
       <c r="M37" s="8"/>
       <c r="N37" s="8"/>
@@ -809,11 +812,11 @@
       <c r="D38" s="7"/>
       <c r="E38" s="8"/>
       <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
+      <c r="G38" s="9"/>
       <c r="H38" s="7"/>
-      <c r="I38" s="9"/>
+      <c r="I38" s="10"/>
       <c r="J38" s="8"/>
-      <c r="K38" s="10"/>
+      <c r="K38" s="11"/>
       <c r="L38" s="8"/>
       <c r="M38" s="8"/>
       <c r="N38" s="8"/>
@@ -829,11 +832,11 @@
       <c r="D39" s="7"/>
       <c r="E39" s="8"/>
       <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
+      <c r="G39" s="9"/>
       <c r="H39" s="7"/>
-      <c r="I39" s="9"/>
+      <c r="I39" s="10"/>
       <c r="J39" s="8"/>
-      <c r="K39" s="10"/>
+      <c r="K39" s="11"/>
       <c r="L39" s="8"/>
       <c r="M39" s="8"/>
       <c r="N39" s="8"/>
@@ -849,11 +852,11 @@
       <c r="D40" s="7"/>
       <c r="E40" s="8"/>
       <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
+      <c r="G40" s="9"/>
       <c r="H40" s="7"/>
-      <c r="I40" s="9"/>
+      <c r="I40" s="10"/>
       <c r="J40" s="8"/>
-      <c r="K40" s="10"/>
+      <c r="K40" s="11"/>
       <c r="L40" s="8"/>
       <c r="M40" s="8"/>
       <c r="N40" s="8"/>
@@ -908,7 +911,7 @@
       </c>
     </row>
     <row r="2" ht="49" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Diese Datei ist die Vorlage für den Förderplan eines Bedarfs aus der Bedarfsliste (Fundraising, Malteser Hilfsdienst e. V., Diözese Paderborn). Sie wird von Hand oder von Copilot ausgefüllt und danach in der Bedarfsliste über „Excel übernehmen“ eingelesen. Der Bedarf mit Summe und noch offenem Betrag steht oben im Blatt „Förderplan“.</t>
         </is>
@@ -916,28 +919,28 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Auftrag</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Finde Förderer, die zu diesem Bedarf passen: Stiftungen, Sparkassen und Volksbanken, Unternehmen, Soziallotterien sowie öffentliche und kirchliche Förderprogramme. Förderer mit Bezug zum Erzbistum Paderborn und zu NRW zuerst, danach bundesweit.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="49" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">2. Recherchiere im Web und prüfe jeden Förderer auf seinen eigenen Seiten: Satzungszweck, Förderrichtlinien, Antragsfristen, übliche Förderhöhe, geforderter Eigenanteil und Antragsweg. Trage als Quellen nur Links ein, die du dabei tatsächlich geöffnet hast. Wenn du nicht im Web suchen kannst, brich ab und sag es mir.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">3. Förderer, die im Blatt „Förderplan“ schon stehen, nicht doppelt anlegen. Steht dort „zugesagt“ oder „abgelehnt“, die Zeile nicht ändern; sonst nur leere Zellen ergänzen.</t>
         </is>
@@ -945,14 +948,14 @@
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Umfang</t>
         </is>
       </c>
     </row>
     <row r="10" ht="49" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">5 bis 8 Förderer, sortiert nach Erfolgsaussicht. Die erwartete Summe je Förderer realistisch aus Förderhistorie, Richtlinien oder üblicher Förderhöhe ableiten; geht das nicht, die Zelle leer lassen. Nicht auf eine Gesamtsumme hinrechnen. Lieber weniger Förderer mit Beleg als viele unsichere.</t>
         </is>
@@ -960,63 +963,63 @@
     </row>
     <row r="11"/>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Regeln</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Je Förderer genau eine Zeile im Blatt „Förderplan“, ab der Zeile unter den Überschriften.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Spaltenüberschriften, Blattnamen und die Angaben oben (Bedarf, Kennung) nicht ändern.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Datum immer als TT.MM.JJJJ, Beträge nur als Zahl in Euro (ohne Text).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Art, Antragsweg und Einschätzung aus der Auswahlliste der Zelle wählen.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Kontakte: bis zu drei Personen, je Person eine Zeile in der Zelle „Name; Funktion; E-Mail; Telefon“.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Kurze Felder kurz halten: „Übliche Fördersumme“ und „Eigenanteil gefordert“ höchstens etwa 80 Zeichen – Erläuterungen gehören in „Notizen“.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Quellen: je Link eine eigene Zeile in der Zelle, nur die Adresse.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">• Unsicheres als solches kennzeichnen (z. B. „laut Website 2025, nicht bestätigt“). Nichts erfinden: lieber eine Zelle leer lassen.</t>
         </is>
@@ -1036,7 +1039,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Förderer</t>
         </is>
@@ -1048,7 +1051,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Stand in der Bedarfsliste</t>
         </is>
@@ -1060,7 +1063,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Art</t>
         </is>
@@ -1072,7 +1075,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Antragsweg</t>
         </is>
@@ -1084,7 +1087,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Kontakte</t>
         </is>
@@ -1096,7 +1099,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">E-Mail</t>
         </is>
@@ -1108,7 +1111,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Telefon</t>
         </is>
@@ -1120,7 +1123,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Website oder Portal-Link</t>
         </is>
@@ -1132,7 +1135,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Antragsfrist</t>
         </is>
@@ -1144,7 +1147,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Weitere Fristen und Termine</t>
         </is>
@@ -1156,7 +1159,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Erwartete Summe (€)</t>
         </is>
@@ -1168,7 +1171,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Übliche Fördersumme</t>
         </is>
@@ -1180,7 +1183,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Eigenanteil gefordert</t>
         </is>
@@ -1192,7 +1195,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Pro – warum passt das?</t>
         </is>
@@ -1204,7 +1207,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Contra – Knackpunkte</t>
         </is>
@@ -1216,7 +1219,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Einschätzung</t>
         </is>
@@ -1228,7 +1231,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Quellen</t>
         </is>
@@ -1240,7 +1243,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Notizen</t>
         </is>

</xml_diff>

<commit_message>
Bedarfsliste 0.42: Copilot als Standard, Cowork nur für die Förderrecherche
- Copilot-Prompt mit festem Antwortblock (#BESCHREIBUNG, #FÖRDERER,
  #KONTAKTE), der in die Liste eingefügt und mit Vorschau übernommen wird
- Cowork nur bei Förderrecherche: ausführliche Word-Datei je Förderer,
  in der Liste nur die Essenz und der Dateiname (neue Spalte/Feld)
- Vorhandenes Pro/Contra wird geprüft und gekürzt
- Auswahl grau → schwarz statt rot

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -175,6 +175,7 @@
     <col min="16" max="16" width="22" customWidth="1"/>
     <col min="17" max="17" width="36" customWidth="1"/>
     <col min="18" max="18" width="30" customWidth="1"/>
+    <col min="19" max="19" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -362,6 +363,11 @@
       <c r="R15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Notizen</t>
+        </is>
+      </c>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ausführliche Recherche (Datei)</t>
         </is>
       </c>
     </row>
@@ -384,6 +390,7 @@
       <c r="P16" s="7"/>
       <c r="Q16" s="8"/>
       <c r="R16" s="8"/>
+      <c r="S16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7"/>
@@ -404,6 +411,7 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="8"/>
       <c r="R17" s="8"/>
+      <c r="S17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7"/>
@@ -424,6 +432,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="8"/>
       <c r="R18" s="8"/>
+      <c r="S18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7"/>
@@ -444,6 +453,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="8"/>
       <c r="R19" s="8"/>
+      <c r="S19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7"/>
@@ -464,6 +474,7 @@
       <c r="P20" s="7"/>
       <c r="Q20" s="8"/>
       <c r="R20" s="8"/>
+      <c r="S20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7"/>
@@ -484,6 +495,7 @@
       <c r="P21" s="7"/>
       <c r="Q21" s="8"/>
       <c r="R21" s="8"/>
+      <c r="S21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7"/>
@@ -504,6 +516,7 @@
       <c r="P22" s="7"/>
       <c r="Q22" s="8"/>
       <c r="R22" s="8"/>
+      <c r="S22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7"/>
@@ -524,6 +537,7 @@
       <c r="P23" s="7"/>
       <c r="Q23" s="8"/>
       <c r="R23" s="8"/>
+      <c r="S23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7"/>
@@ -544,6 +558,7 @@
       <c r="P24" s="7"/>
       <c r="Q24" s="8"/>
       <c r="R24" s="8"/>
+      <c r="S24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7"/>
@@ -564,6 +579,7 @@
       <c r="P25" s="7"/>
       <c r="Q25" s="8"/>
       <c r="R25" s="8"/>
+      <c r="S25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7"/>
@@ -584,6 +600,7 @@
       <c r="P26" s="7"/>
       <c r="Q26" s="8"/>
       <c r="R26" s="8"/>
+      <c r="S26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7"/>
@@ -604,6 +621,7 @@
       <c r="P27" s="7"/>
       <c r="Q27" s="8"/>
       <c r="R27" s="8"/>
+      <c r="S27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7"/>
@@ -624,6 +642,7 @@
       <c r="P28" s="7"/>
       <c r="Q28" s="8"/>
       <c r="R28" s="8"/>
+      <c r="S28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7"/>
@@ -644,6 +663,7 @@
       <c r="P29" s="7"/>
       <c r="Q29" s="8"/>
       <c r="R29" s="8"/>
+      <c r="S29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7"/>
@@ -664,6 +684,7 @@
       <c r="P30" s="7"/>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
+      <c r="S30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7"/>
@@ -684,6 +705,7 @@
       <c r="P31" s="7"/>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
+      <c r="S31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7"/>
@@ -704,6 +726,7 @@
       <c r="P32" s="7"/>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
+      <c r="S32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7"/>
@@ -724,6 +747,7 @@
       <c r="P33" s="7"/>
       <c r="Q33" s="8"/>
       <c r="R33" s="8"/>
+      <c r="S33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7"/>
@@ -744,6 +768,7 @@
       <c r="P34" s="7"/>
       <c r="Q34" s="8"/>
       <c r="R34" s="8"/>
+      <c r="S34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7"/>
@@ -764,6 +789,7 @@
       <c r="P35" s="7"/>
       <c r="Q35" s="8"/>
       <c r="R35" s="8"/>
+      <c r="S35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7"/>
@@ -784,6 +810,7 @@
       <c r="P36" s="7"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="8"/>
+      <c r="S36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7"/>
@@ -804,6 +831,7 @@
       <c r="P37" s="7"/>
       <c r="Q37" s="8"/>
       <c r="R37" s="8"/>
+      <c r="S37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7"/>
@@ -824,6 +852,7 @@
       <c r="P38" s="7"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8"/>
+      <c r="S38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7"/>
@@ -844,6 +873,7 @@
       <c r="P39" s="7"/>
       <c r="Q39" s="8"/>
       <c r="R39" s="8"/>
+      <c r="S39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7"/>
@@ -864,11 +894,12 @@
       <c r="P40" s="7"/>
       <c r="Q40" s="8"/>
       <c r="R40" s="8"/>
+      <c r="S40" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A2:S2"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
@@ -1254,6 +1285,18 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ausführliche Recherche (Datei)</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name der Word-Datei mit der ausführlichen Förderrecherche zu diesem Förderer (im Ordner des Bedarfs), z. B. „Förderrecherche – Sparkasse Paderborn.docx“.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Bedarfsliste 0.43: Ordner finden, kürzere Beschreibung, Ablage je Bedarf
- Kachel „Ordner finden“: Copilot sucht den SharePoint-Ordner (#ORDNER)
- Beschreibung höchstens zwei Absätze, nichts Doppeltes aus der Liste
- Recherche-Dateien ohne Bedarfsordner in einem Unterordner je Bedarf
- Förderersuche: ganzes Gebiet des Erzbistums Paderborn

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6pUX4DTkvdg32w9TEVh4i
</commit_message>
<xml_diff>
--- a/bedarfsliste-app/Foerderplan_Vorlage.xlsx
+++ b/bedarfsliste-app/Foerderplan_Vorlage.xlsx
@@ -956,10 +956,10 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="49" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Finde Förderer, die zu diesem Bedarf passen: Stiftungen, Sparkassen und Volksbanken, Unternehmen, Soziallotterien sowie öffentliche und kirchliche Förderprogramme. Förderer mit Bezug zum Erzbistum Paderborn und zu NRW zuerst, danach bundesweit.</t>
+          <t xml:space="preserve">1. Finde Förderer, die zu diesem Bedarf passen: Stiftungen, Sparkassen und Volksbanken, Unternehmen, Soziallotterien sowie öffentliche und kirchliche Förderprogramme. Förderer mit Bezug zum ganzen Gebiet des Erzbistums Paderborn (z. B. Paderborn, Dortmund, Hagen, Siegen, Höxter) und zu NRW zuerst, danach bundesweit.</t>
         </is>
       </c>
     </row>

</xml_diff>